<commit_message>
Initial upload of complete JKC_v10 project files and dashboards
</commit_message>
<xml_diff>
--- a/AJA/Rohan/Backend/Output/PJPA24_Generated.xlsx
+++ b/AJA/Rohan/Backend/Output/PJPA24_Generated.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2022" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2229" uniqueCount="128">
   <si>
     <t xml:space="preserve">Insight ID </t>
   </si>
@@ -334,21 +334,42 @@
     <t>. Anwar</t>
   </si>
   <si>
+    <t>. Ritesh</t>
+  </si>
+  <si>
+    <t>Boarding without Tax</t>
+  </si>
+  <si>
     <t>4F57434AD60F4190A827</t>
   </si>
   <si>
+    <t>9EDE3B5EC41B46989C30</t>
+  </si>
+  <si>
     <t>13000432</t>
   </si>
   <si>
+    <t>13002169</t>
+  </si>
+  <si>
     <t>05ME3X</t>
   </si>
   <si>
+    <t>6NIN45</t>
+  </si>
+  <si>
     <t>2025-09-10T22:24:59.937</t>
   </si>
   <si>
+    <t>2025-09-09T14:01:43.577</t>
+  </si>
+  <si>
     <t>., Anwar</t>
   </si>
   <si>
+    <t>., Ritesh</t>
+  </si>
+  <si>
     <t>Local Conveyance (Within City)</t>
   </si>
   <si>
@@ -362,6 +383,12 @@
   </si>
   <si>
     <t>Report Date Modified Z-Score (&gt;3.5)</t>
+  </si>
+  <si>
+    <t>Hisar</t>
+  </si>
+  <si>
+    <t>Sirsa</t>
   </si>
   <si>
     <t>8</t>
@@ -2275,7 +2302,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:32">
@@ -2291,7 +2318,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -2299,7 +2326,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -2495,7 +2522,203 @@
         <v>59</v>
       </c>
       <c r="AF7">
-        <v>10.5</v>
+        <v>10.92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H8" s="1">
+        <v>45890</v>
+      </c>
+      <c r="I8">
+        <v>13593.48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>120</v>
+      </c>
+      <c r="K8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8">
+        <v>3000.48</v>
+      </c>
+      <c r="M8" t="s">
+        <v>108</v>
+      </c>
+      <c r="N8" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8">
+        <v>13002169</v>
+      </c>
+      <c r="P8" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>106</v>
+      </c>
+      <c r="R8" t="s">
+        <v>110</v>
+      </c>
+      <c r="S8" t="s">
+        <v>112</v>
+      </c>
+      <c r="T8" t="s">
+        <v>114</v>
+      </c>
+      <c r="U8" t="s">
+        <v>56</v>
+      </c>
+      <c r="V8" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W8" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X8" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y8">
+        <v>13593.48</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA8">
+        <v>13593.48</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD8">
+        <v>13593.48</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF8">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32">
+      <c r="A9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H9" s="1">
+        <v>45891</v>
+      </c>
+      <c r="I9">
+        <v>13593.48</v>
+      </c>
+      <c r="J9" t="s">
+        <v>121</v>
+      </c>
+      <c r="K9" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9">
+        <v>2464</v>
+      </c>
+      <c r="M9" t="s">
+        <v>108</v>
+      </c>
+      <c r="N9" t="s">
+        <v>67</v>
+      </c>
+      <c r="O9">
+        <v>13002169</v>
+      </c>
+      <c r="P9" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>106</v>
+      </c>
+      <c r="R9" t="s">
+        <v>110</v>
+      </c>
+      <c r="S9" t="s">
+        <v>112</v>
+      </c>
+      <c r="T9" t="s">
+        <v>114</v>
+      </c>
+      <c r="U9" t="s">
+        <v>56</v>
+      </c>
+      <c r="V9" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W9" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X9" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y9">
+        <v>13593.48</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA9">
+        <v>13593.48</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD9">
+        <v>13593.48</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF9">
+        <v>3.03</v>
       </c>
     </row>
   </sheetData>
@@ -4979,7 +5202,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF19"/>
+  <dimension ref="A1:AF20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:32">
@@ -5115,7 +5338,7 @@
         <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
         <v>56</v>
@@ -5139,7 +5362,7 @@
         <v>830</v>
       </c>
       <c r="M7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N7" t="s">
         <v>67</v>
@@ -5151,16 +5374,16 @@
         <v>44</v>
       </c>
       <c r="Q7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T7" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U7" t="s">
         <v>56</v>
@@ -5187,7 +5410,7 @@
         <v>87</v>
       </c>
       <c r="AC7" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD7">
         <v>16940</v>
@@ -5196,7 +5419,7 @@
         <v>92</v>
       </c>
       <c r="AF7">
-        <v>5.73</v>
+        <v>5.59</v>
       </c>
     </row>
     <row r="8" spans="1:32">
@@ -5210,7 +5433,7 @@
         <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
         <v>56</v>
@@ -5234,7 +5457,7 @@
         <v>780</v>
       </c>
       <c r="M8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N8" t="s">
         <v>67</v>
@@ -5246,16 +5469,16 @@
         <v>44</v>
       </c>
       <c r="Q8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T8" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U8" t="s">
         <v>56</v>
@@ -5282,7 +5505,7 @@
         <v>87</v>
       </c>
       <c r="AC8" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD8">
         <v>16940</v>
@@ -5291,7 +5514,7 @@
         <v>92</v>
       </c>
       <c r="AF8">
-        <v>5.24</v>
+        <v>5.11</v>
       </c>
     </row>
     <row r="9" spans="1:32">
@@ -5305,7 +5528,7 @@
         <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
         <v>56</v>
@@ -5329,7 +5552,7 @@
         <v>700</v>
       </c>
       <c r="M9" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N9" t="s">
         <v>67</v>
@@ -5341,16 +5564,16 @@
         <v>44</v>
       </c>
       <c r="Q9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R9" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U9" t="s">
         <v>56</v>
@@ -5377,7 +5600,7 @@
         <v>87</v>
       </c>
       <c r="AC9" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD9">
         <v>16940</v>
@@ -5386,7 +5609,7 @@
         <v>92</v>
       </c>
       <c r="AF9">
-        <v>4.44</v>
+        <v>4.34</v>
       </c>
     </row>
     <row r="10" spans="1:32">
@@ -5668,7 +5891,7 @@
         <v>92</v>
       </c>
       <c r="AF12">
-        <v>11.29</v>
+        <v>10.98</v>
       </c>
     </row>
     <row r="13" spans="1:32">
@@ -5760,7 +5983,7 @@
         <v>92</v>
       </c>
       <c r="AF13">
-        <v>8.109999999999999</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="14" spans="1:32">
@@ -5852,7 +6075,7 @@
         <v>92</v>
       </c>
       <c r="AF14">
-        <v>8.109999999999999</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="15" spans="1:32">
@@ -6039,7 +6262,7 @@
         <v>92</v>
       </c>
       <c r="AF16">
-        <v>9.300000000000001</v>
+        <v>9.06</v>
       </c>
     </row>
     <row r="17" spans="1:32">
@@ -6131,7 +6354,7 @@
         <v>92</v>
       </c>
       <c r="AF17">
-        <v>11.39</v>
+        <v>11.08</v>
       </c>
     </row>
     <row r="18" spans="1:32">
@@ -6324,7 +6547,102 @@
         <v>92</v>
       </c>
       <c r="AF19">
-        <v>4.32</v>
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H20" s="1">
+        <v>45891</v>
+      </c>
+      <c r="I20">
+        <v>13593.48</v>
+      </c>
+      <c r="K20" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20">
+        <v>672</v>
+      </c>
+      <c r="M20" t="s">
+        <v>108</v>
+      </c>
+      <c r="N20" t="s">
+        <v>67</v>
+      </c>
+      <c r="O20">
+        <v>13002169</v>
+      </c>
+      <c r="P20" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>106</v>
+      </c>
+      <c r="R20" t="s">
+        <v>110</v>
+      </c>
+      <c r="S20" t="s">
+        <v>112</v>
+      </c>
+      <c r="T20" t="s">
+        <v>114</v>
+      </c>
+      <c r="U20" t="s">
+        <v>56</v>
+      </c>
+      <c r="V20" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W20" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X20" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y20">
+        <v>13593.48</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA20">
+        <v>13593.48</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD20">
+        <v>13593.48</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF20">
+        <v>4.07</v>
       </c>
     </row>
   </sheetData>
@@ -6350,7 +6668,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -6358,7 +6676,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -6548,7 +6866,7 @@
         <v>92</v>
       </c>
       <c r="AF7">
-        <v>4.49</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:32">
@@ -6640,7 +6958,7 @@
         <v>92</v>
       </c>
       <c r="AF8">
-        <v>3.11</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="9" spans="1:32">
@@ -6732,7 +7050,7 @@
         <v>92</v>
       </c>
       <c r="AF9">
-        <v>3.11</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="10" spans="1:32">
@@ -6824,7 +7142,7 @@
         <v>92</v>
       </c>
       <c r="AF10">
-        <v>3.63</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="11" spans="1:32">
@@ -6916,7 +7234,7 @@
         <v>92</v>
       </c>
       <c r="AF11">
-        <v>4.53</v>
+        <v>5.05</v>
       </c>
     </row>
   </sheetData>
@@ -6926,7 +7244,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF19"/>
+  <dimension ref="A1:AF22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:32">
@@ -6942,7 +7260,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -6950,7 +7268,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -7062,7 +7380,7 @@
         <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
         <v>56</v>
@@ -7086,7 +7404,7 @@
         <v>830</v>
       </c>
       <c r="M7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N7" t="s">
         <v>67</v>
@@ -7098,16 +7416,16 @@
         <v>44</v>
       </c>
       <c r="Q7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T7" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U7" t="s">
         <v>56</v>
@@ -7134,7 +7452,7 @@
         <v>87</v>
       </c>
       <c r="AC7" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD7">
         <v>16940</v>
@@ -7157,7 +7475,7 @@
         <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
         <v>56</v>
@@ -7181,7 +7499,7 @@
         <v>780</v>
       </c>
       <c r="M8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N8" t="s">
         <v>67</v>
@@ -7193,16 +7511,16 @@
         <v>44</v>
       </c>
       <c r="Q8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T8" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U8" t="s">
         <v>56</v>
@@ -7229,7 +7547,7 @@
         <v>87</v>
       </c>
       <c r="AC8" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD8">
         <v>16940</v>
@@ -7252,7 +7570,7 @@
         <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
         <v>56</v>
@@ -7276,7 +7594,7 @@
         <v>700</v>
       </c>
       <c r="M9" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N9" t="s">
         <v>67</v>
@@ -7288,16 +7606,16 @@
         <v>44</v>
       </c>
       <c r="Q9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R9" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U9" t="s">
         <v>56</v>
@@ -7324,7 +7642,7 @@
         <v>87</v>
       </c>
       <c r="AC9" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD9">
         <v>16940</v>
@@ -8272,6 +8590,297 @@
       </c>
       <c r="AF19">
         <v>3.79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H20" s="1">
+        <v>45891</v>
+      </c>
+      <c r="I20">
+        <v>13593.48</v>
+      </c>
+      <c r="K20" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20">
+        <v>672</v>
+      </c>
+      <c r="M20" t="s">
+        <v>108</v>
+      </c>
+      <c r="N20" t="s">
+        <v>67</v>
+      </c>
+      <c r="O20">
+        <v>13002169</v>
+      </c>
+      <c r="P20" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>106</v>
+      </c>
+      <c r="R20" t="s">
+        <v>110</v>
+      </c>
+      <c r="S20" t="s">
+        <v>112</v>
+      </c>
+      <c r="T20" t="s">
+        <v>114</v>
+      </c>
+      <c r="U20" t="s">
+        <v>56</v>
+      </c>
+      <c r="V20" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W20" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X20" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y20">
+        <v>13593.48</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA20">
+        <v>13593.48</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD20">
+        <v>13593.48</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF20">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:32">
+      <c r="A21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" t="s">
+        <v>57</v>
+      </c>
+      <c r="G21" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H21" s="1">
+        <v>45890</v>
+      </c>
+      <c r="I21">
+        <v>13593.48</v>
+      </c>
+      <c r="J21" t="s">
+        <v>120</v>
+      </c>
+      <c r="K21" t="s">
+        <v>60</v>
+      </c>
+      <c r="L21">
+        <v>3000.48</v>
+      </c>
+      <c r="M21" t="s">
+        <v>108</v>
+      </c>
+      <c r="N21" t="s">
+        <v>67</v>
+      </c>
+      <c r="O21">
+        <v>13002169</v>
+      </c>
+      <c r="P21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>106</v>
+      </c>
+      <c r="R21" t="s">
+        <v>110</v>
+      </c>
+      <c r="S21" t="s">
+        <v>112</v>
+      </c>
+      <c r="T21" t="s">
+        <v>114</v>
+      </c>
+      <c r="U21" t="s">
+        <v>56</v>
+      </c>
+      <c r="V21" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W21" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X21" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y21">
+        <v>13593.48</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA21">
+        <v>13593.48</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD21">
+        <v>13593.48</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF21">
+        <v>23.78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:32">
+      <c r="A22" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G22" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H22" s="1">
+        <v>45891</v>
+      </c>
+      <c r="I22">
+        <v>13593.48</v>
+      </c>
+      <c r="J22" t="s">
+        <v>121</v>
+      </c>
+      <c r="K22" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22">
+        <v>2464</v>
+      </c>
+      <c r="M22" t="s">
+        <v>108</v>
+      </c>
+      <c r="N22" t="s">
+        <v>67</v>
+      </c>
+      <c r="O22">
+        <v>13002169</v>
+      </c>
+      <c r="P22" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>106</v>
+      </c>
+      <c r="R22" t="s">
+        <v>110</v>
+      </c>
+      <c r="S22" t="s">
+        <v>112</v>
+      </c>
+      <c r="T22" t="s">
+        <v>114</v>
+      </c>
+      <c r="U22" t="s">
+        <v>56</v>
+      </c>
+      <c r="V22" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W22" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X22" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y22">
+        <v>13593.48</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA22">
+        <v>13593.48</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD22">
+        <v>13593.48</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF22">
+        <v>19.15</v>
       </c>
     </row>
   </sheetData>
@@ -8281,7 +8890,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF7"/>
+  <dimension ref="A1:AF8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:32">
@@ -8297,7 +8906,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -8305,7 +8914,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -8501,7 +9110,105 @@
         <v>59</v>
       </c>
       <c r="AF7">
-        <v>9.9</v>
+        <v>10.44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32">
+      <c r="A8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E8" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H8" s="1">
+        <v>45890</v>
+      </c>
+      <c r="I8">
+        <v>13593.48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>120</v>
+      </c>
+      <c r="K8" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8">
+        <v>3000.48</v>
+      </c>
+      <c r="M8" t="s">
+        <v>108</v>
+      </c>
+      <c r="N8" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8">
+        <v>13002169</v>
+      </c>
+      <c r="P8" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>106</v>
+      </c>
+      <c r="R8" t="s">
+        <v>110</v>
+      </c>
+      <c r="S8" t="s">
+        <v>112</v>
+      </c>
+      <c r="T8" t="s">
+        <v>114</v>
+      </c>
+      <c r="U8" t="s">
+        <v>56</v>
+      </c>
+      <c r="V8" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W8" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X8" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y8">
+        <v>13593.48</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA8">
+        <v>13593.48</v>
+      </c>
+      <c r="AB8" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD8">
+        <v>13593.48</v>
+      </c>
+      <c r="AE8" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF8">
+        <v>3.64</v>
       </c>
     </row>
   </sheetData>
@@ -8511,7 +9218,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AF19"/>
+  <dimension ref="A1:AF22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:32">
@@ -8527,7 +9234,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:32">
@@ -8535,7 +9242,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:32">
@@ -8647,7 +9354,7 @@
         <v>97</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
         <v>56</v>
@@ -8671,7 +9378,7 @@
         <v>830</v>
       </c>
       <c r="M7" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N7" t="s">
         <v>67</v>
@@ -8683,16 +9390,16 @@
         <v>44</v>
       </c>
       <c r="Q7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R7" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T7" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U7" t="s">
         <v>56</v>
@@ -8719,7 +9426,7 @@
         <v>87</v>
       </c>
       <c r="AC7" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD7">
         <v>16940</v>
@@ -8728,7 +9435,7 @@
         <v>92</v>
       </c>
       <c r="AF7">
-        <v>4.89</v>
+        <v>5.02</v>
       </c>
     </row>
     <row r="8" spans="1:32">
@@ -8742,7 +9449,7 @@
         <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
         <v>56</v>
@@ -8766,7 +9473,7 @@
         <v>780</v>
       </c>
       <c r="M8" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N8" t="s">
         <v>67</v>
@@ -8778,16 +9485,16 @@
         <v>44</v>
       </c>
       <c r="Q8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R8" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T8" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U8" t="s">
         <v>56</v>
@@ -8814,7 +9521,7 @@
         <v>87</v>
       </c>
       <c r="AC8" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD8">
         <v>16940</v>
@@ -8823,7 +9530,7 @@
         <v>92</v>
       </c>
       <c r="AF8">
-        <v>4.47</v>
+        <v>4.58</v>
       </c>
     </row>
     <row r="9" spans="1:32">
@@ -8837,7 +9544,7 @@
         <v>97</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
         <v>56</v>
@@ -8861,7 +9568,7 @@
         <v>700</v>
       </c>
       <c r="M9" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="N9" t="s">
         <v>67</v>
@@ -8873,16 +9580,16 @@
         <v>44</v>
       </c>
       <c r="Q9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="R9" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="S9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="T9" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="U9" t="s">
         <v>56</v>
@@ -8909,7 +9616,7 @@
         <v>87</v>
       </c>
       <c r="AC9" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="AD9">
         <v>16940</v>
@@ -8918,7 +9625,7 @@
         <v>92</v>
       </c>
       <c r="AF9">
-        <v>3.79</v>
+        <v>3.89</v>
       </c>
     </row>
     <row r="10" spans="1:32">
@@ -9013,7 +9720,7 @@
         <v>58</v>
       </c>
       <c r="AF10">
-        <v>8.210000000000001</v>
+        <v>8.42</v>
       </c>
     </row>
     <row r="11" spans="1:32">
@@ -9108,7 +9815,7 @@
         <v>58</v>
       </c>
       <c r="AF11">
-        <v>8.210000000000001</v>
+        <v>8.42</v>
       </c>
     </row>
     <row r="12" spans="1:32">
@@ -9200,7 +9907,7 @@
         <v>92</v>
       </c>
       <c r="AF12">
-        <v>9.609999999999999</v>
+        <v>9.859999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:32">
@@ -9292,7 +9999,7 @@
         <v>92</v>
       </c>
       <c r="AF13">
-        <v>6.91</v>
+        <v>7.09</v>
       </c>
     </row>
     <row r="14" spans="1:32">
@@ -9384,7 +10091,7 @@
         <v>92</v>
       </c>
       <c r="AF14">
-        <v>6.91</v>
+        <v>7.09</v>
       </c>
     </row>
     <row r="15" spans="1:32">
@@ -9479,7 +10186,7 @@
         <v>58</v>
       </c>
       <c r="AF15">
-        <v>14.04</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="16" spans="1:32">
@@ -9571,7 +10278,7 @@
         <v>92</v>
       </c>
       <c r="AF16">
-        <v>7.93</v>
+        <v>8.130000000000001</v>
       </c>
     </row>
     <row r="17" spans="1:32">
@@ -9663,7 +10370,7 @@
         <v>92</v>
       </c>
       <c r="AF17">
-        <v>9.699999999999999</v>
+        <v>9.94</v>
       </c>
     </row>
     <row r="18" spans="1:32">
@@ -9761,7 +10468,7 @@
         <v>59</v>
       </c>
       <c r="AF18">
-        <v>63.99</v>
+        <v>65.63</v>
       </c>
     </row>
     <row r="19" spans="1:32">
@@ -9856,7 +10563,298 @@
         <v>92</v>
       </c>
       <c r="AF19">
-        <v>3.69</v>
+        <v>3.79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:32">
+      <c r="A20" t="s">
+        <v>103</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>106</v>
+      </c>
+      <c r="E20" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" t="s">
+        <v>57</v>
+      </c>
+      <c r="G20" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H20" s="1">
+        <v>45891</v>
+      </c>
+      <c r="I20">
+        <v>13593.48</v>
+      </c>
+      <c r="K20" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20">
+        <v>672</v>
+      </c>
+      <c r="M20" t="s">
+        <v>108</v>
+      </c>
+      <c r="N20" t="s">
+        <v>67</v>
+      </c>
+      <c r="O20">
+        <v>13002169</v>
+      </c>
+      <c r="P20" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>106</v>
+      </c>
+      <c r="R20" t="s">
+        <v>110</v>
+      </c>
+      <c r="S20" t="s">
+        <v>112</v>
+      </c>
+      <c r="T20" t="s">
+        <v>114</v>
+      </c>
+      <c r="U20" t="s">
+        <v>56</v>
+      </c>
+      <c r="V20" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W20" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X20" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y20">
+        <v>13593.48</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA20">
+        <v>13593.48</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD20">
+        <v>13593.48</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>92</v>
+      </c>
+      <c r="AF20">
+        <v>3.65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:32">
+      <c r="A21" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" t="s">
+        <v>44</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D21" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" t="s">
+        <v>56</v>
+      </c>
+      <c r="F21" t="s">
+        <v>57</v>
+      </c>
+      <c r="G21" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H21" s="1">
+        <v>45890</v>
+      </c>
+      <c r="I21">
+        <v>13593.48</v>
+      </c>
+      <c r="J21" t="s">
+        <v>120</v>
+      </c>
+      <c r="K21" t="s">
+        <v>60</v>
+      </c>
+      <c r="L21">
+        <v>3000.48</v>
+      </c>
+      <c r="M21" t="s">
+        <v>108</v>
+      </c>
+      <c r="N21" t="s">
+        <v>67</v>
+      </c>
+      <c r="O21">
+        <v>13002169</v>
+      </c>
+      <c r="P21" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>106</v>
+      </c>
+      <c r="R21" t="s">
+        <v>110</v>
+      </c>
+      <c r="S21" t="s">
+        <v>112</v>
+      </c>
+      <c r="T21" t="s">
+        <v>114</v>
+      </c>
+      <c r="U21" t="s">
+        <v>56</v>
+      </c>
+      <c r="V21" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W21" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X21" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y21">
+        <v>13593.48</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA21">
+        <v>13593.48</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD21">
+        <v>13593.48</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF21">
+        <v>23.78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:32">
+      <c r="A22" t="s">
+        <v>103</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" t="s">
+        <v>56</v>
+      </c>
+      <c r="F22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G22" s="1">
+        <v>45909</v>
+      </c>
+      <c r="H22" s="1">
+        <v>45891</v>
+      </c>
+      <c r="I22">
+        <v>13593.48</v>
+      </c>
+      <c r="J22" t="s">
+        <v>121</v>
+      </c>
+      <c r="K22" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22">
+        <v>2464</v>
+      </c>
+      <c r="M22" t="s">
+        <v>108</v>
+      </c>
+      <c r="N22" t="s">
+        <v>67</v>
+      </c>
+      <c r="O22">
+        <v>13002169</v>
+      </c>
+      <c r="P22" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>106</v>
+      </c>
+      <c r="R22" t="s">
+        <v>110</v>
+      </c>
+      <c r="S22" t="s">
+        <v>112</v>
+      </c>
+      <c r="T22" t="s">
+        <v>114</v>
+      </c>
+      <c r="U22" t="s">
+        <v>56</v>
+      </c>
+      <c r="V22" s="1">
+        <v>45890</v>
+      </c>
+      <c r="W22" s="1">
+        <v>45892</v>
+      </c>
+      <c r="X22" t="s">
+        <v>85</v>
+      </c>
+      <c r="Y22">
+        <v>13593.48</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA22">
+        <v>13593.48</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>87</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>91</v>
+      </c>
+      <c r="AD22">
+        <v>13593.48</v>
+      </c>
+      <c r="AE22" t="s">
+        <v>121</v>
+      </c>
+      <c r="AF22">
+        <v>19.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>